<commit_message>
chore(commercial): complete objective gate harness
</commit_message>
<xml_diff>
--- a/outputs/commercial-quality/comprehensive-annotated-register.xlsx
+++ b/outputs/commercial-quality/comprehensive-annotated-register.xlsx
@@ -704,6 +704,9 @@
     <t>Effectiveness validation</t>
   </si>
   <si>
+    <t>Failure Response</t>
+  </si>
+  <si>
     <t>Evidence Required</t>
   </si>
   <si>
@@ -740,6 +743,9 @@
     <t>100% of in-scope access reviewed with overdue exceptions escalated.</t>
   </si>
   <si>
+    <t>If the threshold is reached, the process owner records the exception, escalates it to Risk and Audit Committee and tracks closure evidence.</t>
+  </si>
+  <si>
     <t>Current access review export and exception log</t>
   </si>
   <si>
@@ -782,6 +788,9 @@
     <t>All active rules reviewed monthly with stale-rule exceptions tracked.</t>
   </si>
   <si>
+    <t>If the threshold is reached, the process owner records the exception, escalates it to Risk Committee and tracks closure evidence.</t>
+  </si>
+  <si>
     <t>Detection tuning log and rule-change approvals</t>
   </si>
   <si>
@@ -935,10 +944,10 @@
     <t>evidence:EVID-KES-07</t>
   </si>
   <si>
-    <t>Detection rule catalogue, tuning log and alert ageing report</t>
-  </si>
-  <si>
-    <t>Whether the detection rule catalogue, tuning log and alert ageing report demonstrates the stated control condition for the reviewed scope.</t>
+    <t>Detection rule catalogue, tuning log and evidence review record</t>
+  </si>
+  <si>
+    <t>Whether the detection rule catalogue, tuning log and evidence review record demonstrates the stated control condition for the reviewed scope.</t>
   </si>
   <si>
     <t>The condition can create a credible route for loss, delayed detection or weak challenge in operational fraud controls.</t>
@@ -1121,7 +1130,7 @@
     <t>OBS-KES-06</t>
   </si>
   <si>
-    <t>Evidence review: Detection rule catalogue, tuning log and alert ageing report</t>
+    <t>Evidence review: Detection rule catalogue, tuning log and evidence review record</t>
   </si>
   <si>
     <t>OBS-KES-07</t>
@@ -1163,6 +1172,12 @@
     <t>Management Board Decision</t>
   </si>
   <si>
+    <t>Option Analysis</t>
+  </si>
+  <si>
+    <t>Recommendation Rationale</t>
+  </si>
+  <si>
     <t>Approve the Financial Controller mandate for detection ownership and evidence-led oversight.</t>
   </si>
   <si>
@@ -1181,12 +1196,18 @@
     <t>Option A: assign ownership internally; Option B: appoint a specialist partner for the first cycle; Option C: combine internal ownership with targeted specialist validation.</t>
   </si>
   <si>
-    <t>Select the option that gives Financial Controller a named first deliverable, a costed trade-off and a review checkpoint.</t>
+    <t>Select Option B: appoint a specialist partner for the first cycle because it gives Financial Controller a named first deliverable and an independent review checkpoint.</t>
   </si>
   <si>
     <t>Management to confirm Financial Controller as accountable and record the selected option.</t>
   </si>
   <si>
+    <t>Option A: assign ownership internally: cost — Internal management time and process ownership.; benefit — Builds durable internal ownership and operating context.; trade-off — Slower capability uplift while the operating rhythm is established.; rejection reason — Not recommended where immediate independent validation is needed. | Option B: appoint a specialist partner for the first cycle: cost — Specialist fees and a handover dependency.; benefit — Accelerates independent capability and first-cycle delivery.; trade-off — Faster assurance, with recurring cost and dependency on the partner.; recommended option | Option C: combine internal ownership with targeted specialist validation.: cost — Targeted validation cost plus internal coordination time.; benefit — Balances internal accountability with specialist assurance at the decision point.; trade-off — Requires clear boundaries so blended ownership does not dilute accountability.; rejection reason — Not recommended where the organisation cannot fund parallel coordination.</t>
+  </si>
+  <si>
+    <t>This option best balances the stated urgency, control ownership and evidence requirement for Financial Controller.</t>
+  </si>
+  <si>
     <t>MD-KES-01</t>
   </si>
   <si>
@@ -1211,12 +1232,18 @@
     <t>Option A: centralise verification in Accounts Payable; Option B: require business-owner confirmation; Option C: use a bank-validation service with exception review.</t>
   </si>
   <si>
-    <t>Select the option that gives Chief Financial Officer a named first deliverable, a costed trade-off and a review checkpoint.</t>
+    <t>Select Option B: require business-owner confirmation because it gives Chief Financial Officer a named first deliverable and an independent review checkpoint.</t>
   </si>
   <si>
     <t>Management to confirm Chief Financial Officer as accountable and record the selected option.</t>
   </si>
   <si>
+    <t>Option A: centralise verification in Accounts Payable: cost — Internal management time and process ownership.; benefit — Builds durable internal ownership and operating context.; trade-off — Slower capability uplift while the operating rhythm is established.; rejection reason — Not recommended where immediate independent validation is needed. | Option B: require business-owner confirmation: cost — Specialist fees and a handover dependency.; benefit — Accelerates independent capability and first-cycle delivery.; trade-off — Faster assurance, with recurring cost and dependency on the partner.; recommended option | Option C: use a bank-validation service with exception review.: cost — Targeted validation cost plus internal coordination time.; benefit — Balances internal accountability with specialist assurance at the decision point.; trade-off — Requires clear boundaries so blended ownership does not dilute accountability.; rejection reason — Not recommended where the organisation cannot fund parallel coordination.</t>
+  </si>
+  <si>
+    <t>This option best balances the stated urgency, control ownership and evidence requirement for Chief Financial Officer.</t>
+  </si>
+  <si>
     <t>MD-KES-02</t>
   </si>
   <si>
@@ -1232,12 +1259,18 @@
     <t>Option A: close dormant access first; Option B: redesign role profiles first; Option C: run both tracks with weekly exception governance.</t>
   </si>
   <si>
-    <t>Select the option that gives Chief Information Officer a named first deliverable, a costed trade-off and a review checkpoint.</t>
+    <t>Select Option B: redesign role profiles first because it gives Chief Information Officer a named first deliverable and an independent review checkpoint.</t>
   </si>
   <si>
     <t>Management to confirm Chief Information Officer as accountable and record the selected option.</t>
   </si>
   <si>
+    <t>Option A: close dormant access first: cost — Internal management time and process ownership.; benefit — Builds durable internal ownership and operating context.; trade-off — Slower capability uplift while the operating rhythm is established.; rejection reason — Not recommended where immediate independent validation is needed. | Option B: redesign role profiles first: cost — Specialist fees and a handover dependency.; benefit — Accelerates independent capability and first-cycle delivery.; trade-off — Faster assurance, with recurring cost and dependency on the partner.; recommended option | Option C: run both tracks with weekly exception governance.: cost — Targeted validation cost plus internal coordination time.; benefit — Balances internal accountability with specialist assurance at the decision point.; trade-off — Requires clear boundaries so blended ownership does not dilute accountability.; rejection reason — Not recommended where the organisation cannot fund parallel coordination.</t>
+  </si>
+  <si>
+    <t>This option best balances the stated urgency, control ownership and evidence requirement for Chief Information Officer.</t>
+  </si>
+  <si>
     <t>MD-KES-03</t>
   </si>
   <si>
@@ -1253,10 +1286,16 @@
     <t>Option A: strengthen the internal route; Option B: commission an independent channel; Option C: use a blended route with quarterly effectiveness validation.</t>
   </si>
   <si>
-    <t>Select the option that gives Chief People Officer a named first deliverable, a costed trade-off and a review checkpoint.</t>
+    <t>Select Option B: commission an independent channel because it gives Chief People Officer a named first deliverable and an independent review checkpoint.</t>
   </si>
   <si>
     <t>Management to confirm Chief People Officer as accountable and record the selected option.</t>
+  </si>
+  <si>
+    <t>Option A: strengthen the internal route: cost — Internal management time and process ownership.; benefit — Builds durable internal ownership and operating context.; trade-off — Slower capability uplift while the operating rhythm is established.; rejection reason — Not recommended where immediate independent validation is needed. | Option B: commission an independent channel: cost — Specialist fees and a handover dependency.; benefit — Accelerates independent capability and first-cycle delivery.; trade-off — Faster assurance, with recurring cost and dependency on the partner.; recommended option | Option C: use a blended route with quarterly effectiveness validation.: cost — Targeted validation cost plus internal coordination time.; benefit — Balances internal accountability with specialist assurance at the decision point.; trade-off — Requires clear boundaries so blended ownership does not dilute accountability.; rejection reason — Not recommended where the organisation cannot fund parallel coordination.</t>
+  </si>
+  <si>
+    <t>This option best balances the stated urgency, control ownership and evidence requirement for Chief People Officer.</t>
   </si>
   <si>
     <t>MD-KES-04</t>
@@ -2476,45 +2515,48 @@
         <v>229</v>
       </c>
       <c r="N1" t="s">
+        <v>230</v>
+      </c>
+      <c r="O1" t="s">
         <v>65</v>
       </c>
-      <c r="O1" t="s">
-        <v>230</v>
-      </c>
       <c r="P1" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q1" t="s">
         <v>71</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>231</v>
       </c>
       <c r="R1" t="s">
         <v>232</v>
       </c>
       <c r="S1" t="s">
+        <v>233</v>
+      </c>
+      <c r="T1" t="s">
         <v>72</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F2" t="s">
         <v>176</v>
@@ -2529,63 +2571,66 @@
         <v>83</v>
       </c>
       <c r="J2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="P2" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="Q2" t="s">
+        <v>245</v>
+      </c>
+      <c r="R2" t="s">
         <v>84</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>182</v>
       </c>
-      <c r="S2" t="s">
-        <v>244</v>
-      </c>
       <c r="T2" t="s">
-        <v>86</v>
+        <v>246</v>
       </c>
       <c r="U2" t="s">
         <v>86</v>
       </c>
+      <c r="V2" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H3" t="s">
         <v>186</v>
@@ -2594,63 +2639,66 @@
         <v>95</v>
       </c>
       <c r="J3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L3" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="M3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O3" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="P3" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="Q3" t="s">
+        <v>257</v>
+      </c>
+      <c r="R3" t="s">
         <v>96</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>192</v>
       </c>
-      <c r="S3" t="s">
-        <v>255</v>
-      </c>
       <c r="T3" t="s">
-        <v>98</v>
+        <v>258</v>
       </c>
       <c r="U3" t="s">
         <v>98</v>
       </c>
+      <c r="V3" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B4" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C4" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D4" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E4" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F4" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H4" t="s">
         <v>195</v>
@@ -2659,57 +2707,60 @@
         <v>107</v>
       </c>
       <c r="J4" t="s">
+        <v>265</v>
+      </c>
+      <c r="K4" t="s">
+        <v>255</v>
+      </c>
+      <c r="L4" t="s">
+        <v>266</v>
+      </c>
+      <c r="M4" t="s">
+        <v>242</v>
+      </c>
+      <c r="N4" t="s">
+        <v>243</v>
+      </c>
+      <c r="O4" t="s">
+        <v>244</v>
+      </c>
+      <c r="P4" t="s">
         <v>262</v>
       </c>
-      <c r="K4" t="s">
-        <v>263</v>
-      </c>
-      <c r="L4" t="s">
-        <v>240</v>
-      </c>
-      <c r="M4" t="s">
-        <v>241</v>
-      </c>
-      <c r="N4" t="s">
-        <v>242</v>
-      </c>
-      <c r="O4" t="s">
-        <v>259</v>
-      </c>
-      <c r="P4" t="s">
-        <v>264</v>
-      </c>
       <c r="Q4" t="s">
+        <v>267</v>
+      </c>
+      <c r="R4" t="s">
         <v>108</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>199</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>147</v>
-      </c>
-      <c r="T4" t="s">
-        <v>110</v>
       </c>
       <c r="U4" t="s">
         <v>110</v>
       </c>
+      <c r="V4" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F5" t="s">
         <v>176</v>
@@ -2724,63 +2775,66 @@
         <v>83</v>
       </c>
       <c r="J5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O5" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="P5" t="s">
-        <v>265</v>
+        <v>237</v>
       </c>
       <c r="Q5" t="s">
+        <v>268</v>
+      </c>
+      <c r="R5" t="s">
         <v>117</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>205</v>
       </c>
-      <c r="S5" t="s">
-        <v>244</v>
-      </c>
       <c r="T5" t="s">
-        <v>119</v>
+        <v>246</v>
       </c>
       <c r="U5" t="s">
         <v>119</v>
       </c>
+      <c r="V5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H6" t="s">
         <v>186</v>
@@ -2789,63 +2843,66 @@
         <v>95</v>
       </c>
       <c r="J6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L6" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="M6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="P6" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="Q6" t="s">
+        <v>269</v>
+      </c>
+      <c r="R6" t="s">
         <v>124</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>211</v>
       </c>
-      <c r="S6" t="s">
-        <v>255</v>
-      </c>
       <c r="T6" t="s">
-        <v>126</v>
+        <v>258</v>
       </c>
       <c r="U6" t="s">
         <v>126</v>
       </c>
+      <c r="V6" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E7" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H7" t="s">
         <v>195</v>
@@ -2854,57 +2911,60 @@
         <v>107</v>
       </c>
       <c r="J7" t="s">
+        <v>265</v>
+      </c>
+      <c r="K7" t="s">
+        <v>255</v>
+      </c>
+      <c r="L7" t="s">
+        <v>266</v>
+      </c>
+      <c r="M7" t="s">
+        <v>242</v>
+      </c>
+      <c r="N7" t="s">
+        <v>243</v>
+      </c>
+      <c r="O7" t="s">
+        <v>244</v>
+      </c>
+      <c r="P7" t="s">
         <v>262</v>
       </c>
-      <c r="K7" t="s">
-        <v>263</v>
-      </c>
-      <c r="L7" t="s">
-        <v>240</v>
-      </c>
-      <c r="M7" t="s">
-        <v>241</v>
-      </c>
-      <c r="N7" t="s">
-        <v>242</v>
-      </c>
-      <c r="O7" t="s">
-        <v>259</v>
-      </c>
-      <c r="P7" t="s">
-        <v>267</v>
-      </c>
       <c r="Q7" t="s">
+        <v>270</v>
+      </c>
+      <c r="R7" t="s">
         <v>132</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>219</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>147</v>
-      </c>
-      <c r="T7" t="s">
-        <v>134</v>
       </c>
       <c r="U7" t="s">
         <v>134</v>
       </c>
+      <c r="V7" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F8" t="s">
         <v>176</v>
@@ -2919,63 +2979,66 @@
         <v>83</v>
       </c>
       <c r="J8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O8" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="P8" t="s">
-        <v>268</v>
+        <v>237</v>
       </c>
       <c r="Q8" t="s">
+        <v>271</v>
+      </c>
+      <c r="R8" t="s">
         <v>139</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>182</v>
       </c>
-      <c r="S8" t="s">
-        <v>244</v>
-      </c>
       <c r="T8" t="s">
-        <v>141</v>
+        <v>246</v>
       </c>
       <c r="U8" t="s">
         <v>141</v>
       </c>
+      <c r="V8" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C9" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D9" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E9" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F9" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H9" t="s">
         <v>186</v>
@@ -2984,39 +3047,42 @@
         <v>95</v>
       </c>
       <c r="J9" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K9" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L9" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="M9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O9" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="P9" t="s">
-        <v>269</v>
+        <v>250</v>
       </c>
       <c r="Q9" t="s">
+        <v>272</v>
+      </c>
+      <c r="R9" t="s">
         <v>146</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>192</v>
       </c>
-      <c r="S9" t="s">
-        <v>255</v>
-      </c>
       <c r="T9" t="s">
+        <v>258</v>
+      </c>
+      <c r="U9" t="s">
         <v>148</v>
       </c>
-      <c r="U9" t="s">
+      <c r="V9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -3029,61 +3095,61 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B1" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C1" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E1" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="G1" t="s">
         <v>150</v>
       </c>
       <c r="H1" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="I1" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="J1" t="s">
         <v>64</v>
       </c>
       <c r="K1" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="L1" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="M1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N1" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="O1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="P1" t="s">
         <v>166</v>
       </c>
       <c r="Q1" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="R1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="S1" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2">
@@ -3091,55 +3157,55 @@
         <v>183</v>
       </c>
       <c r="B2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C2" t="s">
         <v>76</v>
       </c>
       <c r="D2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G2" t="s">
         <v>191</v>
       </c>
       <c r="H2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J2" t="s">
         <v>44</v>
       </c>
       <c r="K2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="L2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="M2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="O2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="P2" t="s">
         <v>191</v>
       </c>
       <c r="Q2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R2" t="s">
         <v>84</v>
       </c>
       <c r="S2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3">
@@ -3147,84 +3213,84 @@
         <v>206</v>
       </c>
       <c r="B3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C3" t="s">
         <v>113</v>
       </c>
       <c r="D3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G3" t="s">
         <v>191</v>
       </c>
       <c r="H3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
       </c>
       <c r="K3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="L3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="M3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="N3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="O3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="P3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="Q3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R3" t="s">
         <v>117</v>
       </c>
       <c r="S3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B4" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C4" t="s">
         <v>137</v>
       </c>
       <c r="D4" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E4" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F4" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G4" t="s">
         <v>191</v>
       </c>
       <c r="H4" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I4" t="s">
         <v>130</v>
@@ -3233,16 +3299,16 @@
         <v>130</v>
       </c>
       <c r="K4" t="s">
+        <v>310</v>
+      </c>
+      <c r="L4" t="s">
         <v>307</v>
       </c>
-      <c r="L4" t="s">
-        <v>304</v>
-      </c>
       <c r="M4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="N4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="O4" t="s">
         <v>130</v>
@@ -3251,101 +3317,101 @@
         <v>181</v>
       </c>
       <c r="Q4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R4" t="s">
         <v>139</v>
       </c>
       <c r="S4" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C5" t="s">
         <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F5" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G5" t="s">
         <v>191</v>
       </c>
       <c r="H5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="I5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K5" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="Q5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R5" t="s">
         <v>84</v>
       </c>
       <c r="S5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B6" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C6" t="s">
         <v>113</v>
       </c>
       <c r="D6" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E6" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F6" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G6" t="s">
         <v>191</v>
       </c>
       <c r="H6" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="I6" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J6" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K6" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="Q6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R6" t="s">
         <v>117</v>
       </c>
       <c r="S6" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7">
@@ -3353,55 +3419,55 @@
         <v>193</v>
       </c>
       <c r="B7" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C7" t="s">
         <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E7" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F7" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G7" t="s">
         <v>181</v>
       </c>
       <c r="H7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I7" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J7" t="s">
         <v>44</v>
       </c>
       <c r="K7" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="L7" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="M7" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="O7" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="P7" t="s">
         <v>191</v>
       </c>
       <c r="Q7" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R7" t="s">
         <v>96</v>
       </c>
       <c r="S7" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8">
@@ -3409,84 +3475,84 @@
         <v>212</v>
       </c>
       <c r="B8" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C8" t="s">
         <v>122</v>
       </c>
       <c r="D8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E8" t="s">
+        <v>327</v>
+      </c>
+      <c r="F8" t="s">
         <v>323</v>
-      </c>
-      <c r="E8" t="s">
-        <v>324</v>
-      </c>
-      <c r="F8" t="s">
-        <v>320</v>
       </c>
       <c r="G8" t="s">
         <v>181</v>
       </c>
       <c r="H8" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I8" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J8" t="s">
         <v>47</v>
       </c>
       <c r="K8" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="L8" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="M8" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="N8" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="O8" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="P8" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="Q8" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R8" t="s">
         <v>124</v>
       </c>
       <c r="S8" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B9" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C9" t="s">
         <v>144</v>
       </c>
       <c r="D9" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E9" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F9" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G9" t="s">
         <v>181</v>
       </c>
       <c r="H9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I9" t="s">
         <v>41</v>
@@ -3495,72 +3561,72 @@
         <v>41</v>
       </c>
       <c r="K9" t="s">
+        <v>333</v>
+      </c>
+      <c r="L9" t="s">
         <v>330</v>
       </c>
-      <c r="L9" t="s">
-        <v>327</v>
-      </c>
       <c r="M9" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="O9" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="P9" t="s">
         <v>181</v>
       </c>
       <c r="Q9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R9" t="s">
         <v>146</v>
       </c>
       <c r="S9" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B10" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C10" t="s">
         <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="E10" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F10" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G10" t="s">
         <v>181</v>
       </c>
       <c r="H10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="I10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K10" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="Q10" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R10" t="s">
         <v>96</v>
       </c>
       <c r="S10" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11">
@@ -3568,55 +3634,55 @@
         <v>200</v>
       </c>
       <c r="B11" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C11" t="s">
         <v>101</v>
       </c>
       <c r="D11" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E11" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F11" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G11" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="H11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J11" t="s">
         <v>44</v>
       </c>
       <c r="K11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="L11" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="M11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="O11" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="P11" t="s">
         <v>191</v>
       </c>
       <c r="Q11" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R11" t="s">
         <v>108</v>
       </c>
       <c r="S11" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12">
@@ -3624,25 +3690,25 @@
         <v>220</v>
       </c>
       <c r="B12" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C12" t="s">
         <v>129</v>
       </c>
       <c r="D12" t="s">
+        <v>345</v>
+      </c>
+      <c r="E12" t="s">
+        <v>346</v>
+      </c>
+      <c r="F12" t="s">
         <v>342</v>
       </c>
-      <c r="E12" t="s">
-        <v>343</v>
-      </c>
-      <c r="F12" t="s">
-        <v>339</v>
-      </c>
       <c r="G12" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="H12" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I12" t="s">
         <v>130</v>
@@ -3651,16 +3717,16 @@
         <v>130</v>
       </c>
       <c r="K12" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="L12" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="M12" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="N12" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="O12" t="s">
         <v>130</v>
@@ -3669,57 +3735,57 @@
         <v>181</v>
       </c>
       <c r="Q12" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R12" t="s">
         <v>132</v>
       </c>
       <c r="S12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C13" t="s">
         <v>101</v>
       </c>
       <c r="D13" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E13" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F13" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G13" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="H13" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="I13" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J13" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K13" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="Q13" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="R13" t="s">
         <v>108</v>
       </c>
       <c r="S13" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -3731,48 +3797,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B1" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C1" t="s">
         <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E1" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F1" t="s">
         <v>71</v>
       </c>
       <c r="G1" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="H1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C2" t="s">
         <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E2" t="s">
         <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="G2" t="s">
         <v>86</v>
@@ -3783,22 +3849,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C3" t="s">
         <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E3" t="s">
         <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="G3" t="s">
         <v>98</v>
@@ -3809,22 +3875,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C4" t="s">
         <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E4" t="s">
         <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G4" t="s">
         <v>110</v>
@@ -3835,22 +3901,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B5" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C5" t="s">
         <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E5" t="s">
         <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G5" t="s">
         <v>119</v>
@@ -3861,22 +3927,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B6" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C6" t="s">
         <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E6" t="s">
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="G6" t="s">
         <v>126</v>
@@ -3887,22 +3953,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B7" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C7" t="s">
         <v>130</v>
       </c>
       <c r="D7" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E7" t="s">
         <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="G7" t="s">
         <v>134</v>
@@ -3913,22 +3979,22 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B8" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C8" t="s">
         <v>130</v>
       </c>
       <c r="D8" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E8" t="s">
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G8" t="s">
         <v>141</v>
@@ -3939,22 +4005,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B9" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E9" t="s">
         <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="G9" t="s">
         <v>148</v>
@@ -3972,209 +4038,239 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B1" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="C1" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D1" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E1" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F1" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G1" t="s">
         <v>70</v>
       </c>
       <c r="H1" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="I1" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="J1" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="K1" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="L1" t="s">
+        <v>383</v>
+      </c>
+      <c r="M1" t="s">
+        <v>384</v>
+      </c>
+      <c r="N1" t="s">
         <v>71</v>
       </c>
-      <c r="M1" t="s">
-        <v>231</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>232</v>
+      </c>
+      <c r="P1" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B2" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C2" t="s">
         <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E2" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="F2" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H2" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="I2" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="J2" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="K2" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="L2" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="M2" t="s">
+        <v>394</v>
+      </c>
+      <c r="N2" t="s">
+        <v>395</v>
+      </c>
+      <c r="O2" t="s">
         <v>84</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B3" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C3" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="D3" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="E3" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="F3" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="H3" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="I3" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="J3" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="K3" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="L3" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="M3" t="s">
+        <v>406</v>
+      </c>
+      <c r="N3" t="s">
+        <v>407</v>
+      </c>
+      <c r="O3" t="s">
         <v>96</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="B4" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
       <c r="C4" t="s">
         <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="E4" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="F4" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="H4" t="s">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="I4" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
       <c r="J4" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
       <c r="K4" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="L4" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="M4" t="s">
+        <v>415</v>
+      </c>
+      <c r="N4" t="s">
+        <v>416</v>
+      </c>
+      <c r="O4" t="s">
         <v>108</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
       <c r="B5" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="C5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D5" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E5" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="F5" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="H5" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="I5" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="J5" t="s">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="K5" t="s">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="L5" t="s">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="M5" t="s">
+        <v>424</v>
+      </c>
+      <c r="N5" t="s">
+        <v>425</v>
+      </c>
+      <c r="O5" t="s">
         <v>117</v>
       </c>
-      <c r="N5" t="s">
+      <c r="P5" t="s">
         <v>205</v>
       </c>
     </row>

</xml_diff>